<commit_message>
Dashboard 2026-08-31 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339104182/spec-339104182.xlsx
+++ b/vse-loti/339104182/spec-339104182.xlsx
@@ -61,14 +61,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -446,8 +448,6 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,25 +478,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Цена за ед. (без НДС)</t>
+          <t>Стоимость (без НДС)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Цена за ед. (с НДС)</t>
+          <t>Цена за т (без НДС)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Стоимость (без НДС)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Цена за т (без НДС)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Цена за т (с НДС)</t>
         </is>
@@ -508,33 +498,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Бензин автомобильный АИ-92</t>
+          <t>Коммерческое предложение № 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>60000</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>л; дм3</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>132</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>132</v>
-      </c>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -542,11 +521,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Бензин автомобильный АИ-95</t>
+          <t>Бензин автомобильный АИ-92</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>20000</v>
+        <v>60000</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -554,21 +533,11 @@
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" s="3" t="n">
-        <v>119</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>142.8</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>2380000</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>119</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>142.8</v>
-      </c>
+      <c r="F3" s="4" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -576,58 +545,75 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Бензин автомобильный АИ-95</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>л; дм3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="4" t="n">
+        <v>2380000</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Дизельное топливо (зимнее)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C5" s="2" t="n">
         <v>30000</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>л; дм3</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="3" t="n">
-        <v>124</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>148.8</v>
-      </c>
-      <c r="H4" s="3" t="n">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="4" t="n">
         <v>3720000</v>
       </c>
-      <c r="I4" s="3" t="n">
-        <v>124</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>148.8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n">
         <v>12700000</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>НМЦК из обоснования:</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="F7" s="7" t="n">
         <v>12700000</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Источник: 1015_Обоснование НМЦД_гсм.xlsx</t>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Источник: 1015Д_ТЗ_ГСМ.docx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard 2026-09-01 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339104182/spec-339104182.xlsx
+++ b/vse-loti/339104182/spec-339104182.xlsx
@@ -16,11 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00&quot; ₽&quot;"/>
-  </numFmts>
-  <fonts count="3">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +26,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF808080"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,7 +49,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
+        <fgColor rgb="FF305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,17 +70,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,17 +458,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,37 +480,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Наименование позиции (⌀ + s, если указано)</t>
+          <t>Наименование позиции</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Характеристика</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Кол-во (исх.)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Масса, т (приведённая)</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Объём, л</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Стоимость (без НДС)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Цена за т (без НДС)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Цена за т (с НДС)</t>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Цена за л (без НДС)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Цена за л (с НДС)</t>
         </is>
       </c>
     </row>
@@ -498,22 +525,34 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Коммерческое предложение № 1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>т</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>Бензин автомобильный АИ-92</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ГОСТ 32513-2023; К5; октановое ≥ 92 и &lt; 95</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>л; дм³</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>91.67</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -521,23 +560,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Бензин автомобильный АИ-92</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>60000</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>л; дм3</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" s="4" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+          <t>Бензин автомобильный АИ-95</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ГОСТ 32513-2023; К5; октановое ≥ 95 и &lt; 98</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>л; дм³</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>1983333.33</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>99.17</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>119</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -545,75 +595,99 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Бензин автомобильный АИ-95</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>л; дм3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="4" t="n">
-        <v>2380000</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+          <t>Дизельное топливо (зимнее)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ГОСТ 32511-2013; К5; сорт/класс ≥ F; зимнее</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>л; дм³</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>103.33</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>124</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Дизельное топливо (зимнее)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>30000</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>л; дм3</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" s="4" t="n">
-        <v>3720000</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="9" t="n">
+        <v>110000</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>10583333.33</v>
+      </c>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="7" t="n">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>НМЦК (без НДС):</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>10583333.33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>НМЦК (с НДС):</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
         <v>12700000</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>НМЦК из обоснования:</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>12700000</v>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Источник: 1015Д_ТЗ_ГСМ.docx</t>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Источник 1 (позиции, цены, кол-во): 1015_Обоснование НМЦД_гсм.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Источник 2 (ОКПД2, ГОСТ, экол. класс): 1015Д_ТЗ_ГСМ.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Источник 3 (НМЦД, формула цены): 1015_Аукцион двухчастный_ГСМ.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Источник 4 (подтверждение «цена с НДС»): 1015Д_Проект договора_ГСМ_по пост оплате.docx</t>
         </is>
       </c>
     </row>

</xml_diff>